<commit_message>
feat(F-NAR-019): TREE-COL-025 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-COL-025.xlsx
+++ b/stories/arbres/TREE-COL-025.xlsx
@@ -854,7 +854,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Sous la pluie, la gouttière de zinc déborde : une feuille coince le coude, et l'eau rate le pot de basilic de Nina. Elle veut le dire tout de suite, mais ses mots se cognent à ceux de papa. Cuisine, jardin ou chambre changent l'obstacle ; cubes, livre ou dînette changent la manière de montrer ; matin, sieste ou soir changent le rythme de l'attente. Quand sa main lève une place, le bol bleu reçoit enfin l'eau, et le zinc chante plus juste.</t>
+          <t>Sous la pluie, la gouttière de zinc déborde : une feuille coince le coude, et l'eau rate le pot de basilic de Nina. Elle veut le dire tout de suite, mais ses mots se cognent à ceux de papa. Cuisine, jardin ou chambre changent l'obstacle ; cubes, livre ou dînette changent la manière de montrer ; matin, sieste ou soir changent le rythme de l'attente. Quand sa main ouvre une place, le bol bleu reçoit enfin l'eau, et le zinc chante plus juste.</t>
         </is>
       </c>
     </row>
@@ -2542,17 +2542,17 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Le petit zinc de cubes peut attendre le matin, après la sieste, ou le soir. Quand montrons-nous la feuille au vrai zinc ?</t>
+          <t>Le petit zinc de cubes peut se montrer le matin, après la sieste, ou le soir. Quand montrons-nous la feuille au vrai zinc ?</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Le petit zinc de cubes peut attendre le matin, après la sieste, ou le soir. Quand montrons-nous la feuille au vrai zinc ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Le petit zinc de cubes peut se montrer le matin, après la sieste, ou le soir. Quand montrons-nous la feuille au vrai zinc ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Le petit zinc de cubes peut attendre le matin, après la sieste, ou le soir. Quand montrons-nous la feuille au vrai zinc ?&lt;/slow&gt; [long-pause]</t>
+          <t>&lt;slow&gt;Le petit zinc de cubes peut se montrer le matin, après la sieste, ou le soir. Quand montrons-nous la feuille au vrai zinc ?&lt;/slow&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr"/>
@@ -2710,7 +2710,7 @@
       </c>
       <c r="AW9" t="inlineStr">
         <is>
-          <t>narrateur|Le petit zinc de cubes peut attendre le matin, après la sieste, ou le soir.
+          <t>narrateur|Le petit zinc de cubes peut se montrer le matin, après la sieste, ou le soir.
 papa|Quand montrons-nous la feuille au vrai zinc ?</t>
         </is>
       </c>
@@ -7218,17 +7218,17 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>La feuille ! Oui, coincée dans le zinc. Maman a vu le doigt, puis le coude. Merci d'avoir attendu le calme. Le vent nous avait mélangés. Montre-nous avec un objet, maintenant.</t>
+          <t>La feuille ! Oui, coincée dans le zinc. Maman a vu le doigt, puis le coude. Merci d'avoir laissé le vent passer. Le vent nous avait mélangés. Montre-nous avec un objet, maintenant.</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La feuille ! Oui, coincée dans le zinc. Maman a vu le doigt, puis le coude. Merci d'avoir attendu le calme. Le vent nous avait mélangés. Montre-nous avec un objet, &lt;emphasis level="moderate"&gt;main&lt;/emphasis&gt;tenant.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La feuille ! Oui, coincée dans le zinc. Maman a vu le doigt, puis le coude. Merci d'avoir laissé le vent passer. Le vent nous avait mélangés. Montre-nous avec un objet, &lt;emphasis level="moderate"&gt;main&lt;/emphasis&gt;tenant.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>La feuille ! Oui, coincée dans le zinc. Maman a vu le doigt, puis le coude. Merci d'avoir attendu le calme. Le vent nous avait mélangés. Montre-nous avec un objet, &lt;emphasis&gt;main&lt;/emphasis&gt;tenant. [pause]</t>
+          <t>La feuille ! Oui, coincée dans le zinc. Maman a vu le doigt, puis le coude. Merci d'avoir laissé le vent passer. Le vent nous avait mélangés. Montre-nous avec un objet, &lt;emphasis&gt;main&lt;/emphasis&gt;tenant. [pause]</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr"/>
@@ -7365,7 +7365,7 @@
           <t>enfant-f|La feuille !
 narrateur|Oui, coincée dans le zinc.
 narrateur|Maman a vu le doigt, puis le coude.
-papa|Merci d'avoir attendu le calme.
+papa|Merci d'avoir laissé le vent passer.
 maman|Le vent nous avait mélangés.
 papa|Montre-nous avec un objet, maintenant.</t>
         </is>
@@ -7788,17 +7788,17 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Les cubes mouillés peuvent attendre le matin, après la sieste, ou le soir. Quand allons-nous au coude ?</t>
+          <t>Les cubes mouillés peuvent servir le matin, après la sieste, ou le soir. Quand allons-nous au coude ?</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Les cubes mouillés peuvent attendre le matin, après la sieste, ou le soir. Quand allons-nous au coude ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Les cubes mouillés peuvent servir le matin, après la sieste, ou le soir. Quand allons-nous au coude ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Les cubes mouillés peuvent attendre le matin, après la sieste, ou le soir. Quand allons-nous au coude ?&lt;/slow&gt; [long-pause]</t>
+          <t>&lt;slow&gt;Les cubes mouillés peuvent servir le matin, après la sieste, ou le soir. Quand allons-nous au coude ?&lt;/slow&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr"/>
@@ -7956,7 +7956,7 @@
       </c>
       <c r="AW37" t="inlineStr">
         <is>
-          <t>narrateur|Les cubes mouillés peuvent attendre le matin, après la sieste, ou le soir.
+          <t>narrateur|Les cubes mouillés peuvent servir le matin, après la sieste, ou le soir.
 maman|Quand allons-nous au coude ?</t>
         </is>
       </c>
@@ -15094,17 +15094,17 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Après la sieste, le livre sert de toit au doudou. Nina lève la main, sans le déranger. Nous t'écoutons. On approche le bol, tout doucement. Le filet lent entre. Ils glissent la feuille comme un signet, un instant. La page a tenu ta place. Nina repose le livre sur le doudou. La chambre est un nid d'écoute.</t>
+          <t>Après la sieste, le livre sert de toit au doudou. Nina lève la main, sans le déranger. Nous t'écoutons. On approche le bol, sans le faire tinter. Le filet lent entre. Ils glissent la feuille comme un signet, un instant. La page a tenu ta place. Nina repose le livre sur le doudou. La chambre est un nid d'écoute.</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Après la sieste, le livre sert de toit au doudou. Nina lève la main, sans le déranger. Nous t'écoutons. On approche le bol, tout doucement. Le filet lent entre. Ils glissent la feuille comme un signet, un instant. La page a tenu ta place. Nina repose le livre sur le doudou. La chambre est un nid d'écoute.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Après la sieste, le livre sert de toit au doudou. Nina lève la main, sans le déranger. Nous t'écoutons. On approche le bol, sans le faire tinter. Le filet lent entre. Ils glissent la feuille comme un signet, un instant. La page a tenu ta place. Nina repose le livre sur le doudou. La chambre est un nid d'écoute.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>Après la sieste, le livre sert de toit au doudou. Nina lève la main, sans le déranger. Nous t'écoutons. On approche le bol, tout doucement. Le filet lent entre. Ils glissent la feuille comme un signet, un instant. La page a tenu ta place. Nina repose le livre sur le doudou. La chambre est un nid d'écoute. [pause]</t>
+          <t>Après la sieste, le livre sert de toit au doudou. Nina lève la main, sans le déranger. Nous t'écoutons. On approche le bol, sans le faire tinter. Le filet lent entre. Ils glissent la feuille comme un signet, un instant. La page a tenu ta place. Nina repose le livre sur le doudou. La chambre est un nid d'écoute. [pause]</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr"/>
@@ -15241,7 +15241,7 @@
           <t>narrateur|Après la sieste, le livre sert de toit au doudou.
 narrateur|Nina lève la main, sans le déranger.
 papa|Nous t'écoutons.
-enfant-f|On approche le bol, tout doucement.
+enfant-f|On approche le bol, sans le faire tinter.
 narrateur|Le filet lent entre.
 narrateur|Ils glissent la feuille comme un signet, un instant.
 maman|La page a tenu ta place.
@@ -16025,17 +16025,17 @@
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>L'assiette naine peut attendre le matin, après la sieste, ou le soir. Quand attrapons-nous la goutte ?</t>
+          <t>L'assiette naine peut travailler le matin, après la sieste, ou le soir. Quand attrapons-nous la goutte ?</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;L'assiette naine peut attendre le matin, après la sieste, ou le soir. Quand attrapons-nous la goutte ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;L'assiette naine peut travailler le matin, après la sieste, ou le soir. Quand attrapons-nous la goutte ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;L'assiette naine peut attendre le matin, après la sieste, ou le soir. Quand attrapons-nous la goutte ?&lt;/slow&gt; [long-pause]</t>
+          <t>&lt;slow&gt;L'assiette naine peut travailler le matin, après la sieste, ou le soir. Quand attrapons-nous la goutte ?&lt;/slow&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr"/>
@@ -16193,7 +16193,7 @@
       </c>
       <c r="AW81" t="inlineStr">
         <is>
-          <t>narrateur|L'assiette naine peut attendre le matin, après la sieste, ou le soir.
+          <t>narrateur|L'assiette naine peut travailler le matin, après la sieste, ou le soir.
 papa|Quand attrapons-nous la goutte ?</t>
         </is>
       </c>
@@ -16405,17 +16405,17 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Le rebord sent l'eau neuve. Raconte la perle. La tasse a visé, le bol a reçu. La tasse naine attrape une goutte du rebord. Le basilic tremble, puis se tient. Nina essuie sa main au rideau, tout doucement.</t>
+          <t>Le rebord sent l'eau neuve. Raconte la perle. La tasse a visé, le bol a reçu. La tasse naine attrape une goutte du rebord. Le basilic tremble, puis se tient. Nina essuie sa main au rideau, sans bruit.</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le rebord sent l'eau neuve. Raconte la perle. La tasse a visé, le bol a reçu. La tasse naine attrape une goutte du rebord. Le basilic tremble, puis se tient. Nina essuie sa &lt;emphasis level="moderate"&gt;main&lt;/emphasis&gt; au rideau, tout doucement.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le rebord sent l'eau neuve. Raconte la perle. La tasse a visé, le bol a reçu. La tasse naine attrape une goutte du rebord. Le basilic tremble, puis se tient. Nina essuie sa &lt;emphasis level="moderate"&gt;main&lt;/emphasis&gt; au rideau, sans bruit.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le rebord sent l'eau neuve. Raconte la perle. La tasse a visé, le bol a reçu. La tasse naine attrape une goutte du rebord. Le basilic tremble, puis se tient. Nina essuie sa &lt;emphasis&gt;main&lt;/emphasis&gt; au rideau, tout doucement.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le rebord sent l'eau neuve. Raconte la perle. La tasse a visé, le bol a reçu. La tasse naine attrape une goutte du rebord. Le basilic tremble, puis se tient. Nina essuie sa &lt;emphasis&gt;main&lt;/emphasis&gt; au rideau, sans bruit.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr"/>
@@ -16558,7 +16558,7 @@
 enfant-f|La tasse a visé, le bol a reçu.
 narrateur|La tasse naine attrape une goutte du rebord.
 narrateur|Le basilic tremble, puis se tient.
-narrateur|Nina essuie sa main au rideau, tout doucement.</t>
+narrateur|Nina essuie sa main au rideau, sans bruit.</t>
         </is>
       </c>
       <c r="AX83" t="inlineStr">
@@ -17322,7 +17322,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17379,6 +17379,13 @@
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>